<commit_message>
Initial commit - Aplikasi KlasterKu
</commit_message>
<xml_diff>
--- a/media/hasil/hasil_clustering_customer.xlsx
+++ b/media/hasil/hasil_clustering_customer.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D183"/>
+  <dimension ref="A1:E183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,6 +434,11 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Frekuensi</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Cluster</t>
         </is>
       </c>
@@ -451,7 +456,10 @@
         <v>22672000000</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>52</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -467,6 +475,9 @@
         <v>10900000</v>
       </c>
       <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -483,7 +494,10 @@
         <v>4579500000</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>69</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -499,6 +513,9 @@
         <v>32700000</v>
       </c>
       <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -515,6 +532,9 @@
         <v>23630000</v>
       </c>
       <c r="D6" t="n">
+        <v>11</v>
+      </c>
+      <c r="E6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -531,6 +551,9 @@
         <v>6867000000</v>
       </c>
       <c r="D7" t="n">
+        <v>21</v>
+      </c>
+      <c r="E7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -547,7 +570,10 @@
         <v>1256700000</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>54</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -563,6 +589,9 @@
         <v>27040000</v>
       </c>
       <c r="D9" t="n">
+        <v>13</v>
+      </c>
+      <c r="E9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -579,6 +608,9 @@
         <v>605450000</v>
       </c>
       <c r="D10" t="n">
+        <v>40</v>
+      </c>
+      <c r="E10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -595,6 +627,9 @@
         <v>2106540000</v>
       </c>
       <c r="D11" t="n">
+        <v>36</v>
+      </c>
+      <c r="E11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -611,7 +646,10 @@
         <v>2265940000</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>106</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -627,6 +665,9 @@
         <v>32700000</v>
       </c>
       <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -643,6 +684,9 @@
         <v>391500000</v>
       </c>
       <c r="D14" t="n">
+        <v>24</v>
+      </c>
+      <c r="E14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -659,6 +703,9 @@
         <v>64980280000</v>
       </c>
       <c r="D15" t="n">
+        <v>73</v>
+      </c>
+      <c r="E15" t="n">
         <v>2</v>
       </c>
     </row>
@@ -675,7 +722,10 @@
         <v>17105500000</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>97</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -691,6 +741,9 @@
         <v>305200000</v>
       </c>
       <c r="D17" t="n">
+        <v>14</v>
+      </c>
+      <c r="E17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -707,6 +760,9 @@
         <v>31950000</v>
       </c>
       <c r="D18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -723,6 +779,9 @@
         <v>223650000</v>
       </c>
       <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -739,7 +798,10 @@
         <v>7896950000</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>57</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -755,6 +817,9 @@
         <v>74550000</v>
       </c>
       <c r="D21" t="n">
+        <v>7</v>
+      </c>
+      <c r="E21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -771,6 +836,9 @@
         <v>2592250000</v>
       </c>
       <c r="D22" t="n">
+        <v>26</v>
+      </c>
+      <c r="E22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -787,6 +855,9 @@
         <v>53250000</v>
       </c>
       <c r="D23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -803,6 +874,9 @@
         <v>32700000</v>
       </c>
       <c r="D24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -819,6 +893,9 @@
         <v>545000000</v>
       </c>
       <c r="D25" t="n">
+        <v>19</v>
+      </c>
+      <c r="E25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -835,6 +912,9 @@
         <v>18560000</v>
       </c>
       <c r="D26" t="n">
+        <v>8</v>
+      </c>
+      <c r="E26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -851,6 +931,9 @@
         <v>933800000</v>
       </c>
       <c r="D27" t="n">
+        <v>32</v>
+      </c>
+      <c r="E27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -867,6 +950,9 @@
         <v>140450000</v>
       </c>
       <c r="D28" t="n">
+        <v>13</v>
+      </c>
+      <c r="E28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -883,6 +969,9 @@
         <v>29967850000</v>
       </c>
       <c r="D29" t="n">
+        <v>226</v>
+      </c>
+      <c r="E29" t="n">
         <v>2</v>
       </c>
     </row>
@@ -899,7 +988,10 @@
         <v>13554200000</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>139</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="31">
@@ -915,6 +1007,9 @@
         <v>1789200000</v>
       </c>
       <c r="D31" t="n">
+        <v>24</v>
+      </c>
+      <c r="E31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -931,6 +1026,9 @@
         <v>130050000</v>
       </c>
       <c r="D32" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -947,6 +1045,9 @@
         <v>852000000</v>
       </c>
       <c r="D33" t="n">
+        <v>8</v>
+      </c>
+      <c r="E33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -963,6 +1064,9 @@
         <v>3814920000</v>
       </c>
       <c r="D34" t="n">
+        <v>49</v>
+      </c>
+      <c r="E34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -979,6 +1083,9 @@
         <v>31950000</v>
       </c>
       <c r="D35" t="n">
+        <v>3</v>
+      </c>
+      <c r="E35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -995,6 +1102,9 @@
         <v>30785050000</v>
       </c>
       <c r="D36" t="n">
+        <v>91</v>
+      </c>
+      <c r="E36" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1011,6 +1121,9 @@
         <v>837600000</v>
       </c>
       <c r="D37" t="n">
+        <v>27</v>
+      </c>
+      <c r="E37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1027,6 +1140,9 @@
         <v>6540000</v>
       </c>
       <c r="D38" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1043,6 +1159,9 @@
         <v>1544700000</v>
       </c>
       <c r="D39" t="n">
+        <v>8</v>
+      </c>
+      <c r="E39" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1059,6 +1178,9 @@
         <v>778800000</v>
       </c>
       <c r="D40" t="n">
+        <v>32</v>
+      </c>
+      <c r="E40" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1075,6 +1197,9 @@
         <v>2672680000</v>
       </c>
       <c r="D41" t="n">
+        <v>43</v>
+      </c>
+      <c r="E41" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1091,6 +1216,9 @@
         <v>654000000</v>
       </c>
       <c r="D42" t="n">
+        <v>3</v>
+      </c>
+      <c r="E42" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1107,6 +1235,9 @@
         <v>76300000</v>
       </c>
       <c r="D43" t="n">
+        <v>7</v>
+      </c>
+      <c r="E43" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1123,6 +1254,9 @@
         <v>545000000</v>
       </c>
       <c r="D44" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1139,6 +1273,9 @@
         <v>32700000</v>
       </c>
       <c r="D45" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1155,7 +1292,10 @@
         <v>3514500000</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>63</v>
+      </c>
+      <c r="E46" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="47">
@@ -1171,6 +1311,9 @@
         <v>218000000</v>
       </c>
       <c r="D47" t="n">
+        <v>5</v>
+      </c>
+      <c r="E47" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1187,6 +1330,9 @@
         <v>2619900000</v>
       </c>
       <c r="D48" t="n">
+        <v>39</v>
+      </c>
+      <c r="E48" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1203,6 +1349,9 @@
         <v>867650000</v>
       </c>
       <c r="D49" t="n">
+        <v>41</v>
+      </c>
+      <c r="E49" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1219,6 +1368,9 @@
         <v>108300000</v>
       </c>
       <c r="D50" t="n">
+        <v>10</v>
+      </c>
+      <c r="E50" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1235,7 +1387,10 @@
         <v>2821100000</v>
       </c>
       <c r="D51" t="n">
-        <v>0</v>
+        <v>70</v>
+      </c>
+      <c r="E51" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="52">
@@ -1251,6 +1406,9 @@
         <v>23856000000</v>
       </c>
       <c r="D52" t="n">
+        <v>42</v>
+      </c>
+      <c r="E52" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1267,6 +1425,9 @@
         <v>1471205000000</v>
       </c>
       <c r="D53" t="n">
+        <v>141</v>
+      </c>
+      <c r="E53" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1283,6 +1444,9 @@
         <v>1169800000</v>
       </c>
       <c r="D54" t="n">
+        <v>42</v>
+      </c>
+      <c r="E54" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1299,6 +1463,9 @@
         <v>2689750000</v>
       </c>
       <c r="D55" t="n">
+        <v>9</v>
+      </c>
+      <c r="E55" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1315,6 +1482,9 @@
         <v>272500000</v>
       </c>
       <c r="D56" t="n">
+        <v>5</v>
+      </c>
+      <c r="E56" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1331,6 +1501,9 @@
         <v>394800000</v>
       </c>
       <c r="D57" t="n">
+        <v>9</v>
+      </c>
+      <c r="E57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1347,6 +1520,9 @@
         <v>117150000</v>
       </c>
       <c r="D58" t="n">
+        <v>11</v>
+      </c>
+      <c r="E58" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1363,6 +1539,9 @@
         <v>457800000</v>
       </c>
       <c r="D59" t="n">
+        <v>3</v>
+      </c>
+      <c r="E59" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1379,6 +1558,9 @@
         <v>213000000</v>
       </c>
       <c r="D60" t="n">
+        <v>5</v>
+      </c>
+      <c r="E60" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1395,6 +1577,9 @@
         <v>397125000</v>
       </c>
       <c r="D61" t="n">
+        <v>38</v>
+      </c>
+      <c r="E61" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1411,6 +1596,9 @@
         <v>37822500000</v>
       </c>
       <c r="D62" t="n">
+        <v>70</v>
+      </c>
+      <c r="E62" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1427,6 +1615,9 @@
         <v>170400000</v>
       </c>
       <c r="D63" t="n">
+        <v>8</v>
+      </c>
+      <c r="E63" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1443,6 +1634,9 @@
         <v>196200000</v>
       </c>
       <c r="D64" t="n">
+        <v>18</v>
+      </c>
+      <c r="E64" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1459,7 +1653,10 @@
         <v>1255800000</v>
       </c>
       <c r="D65" t="n">
-        <v>0</v>
+        <v>114</v>
+      </c>
+      <c r="E65" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="66">
@@ -1475,6 +1672,9 @@
         <v>109000000</v>
       </c>
       <c r="D66" t="n">
+        <v>5</v>
+      </c>
+      <c r="E66" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1491,6 +1691,9 @@
         <v>159750000</v>
       </c>
       <c r="D67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E67" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1507,6 +1710,9 @@
         <v>2556000000</v>
       </c>
       <c r="D68" t="n">
+        <v>3</v>
+      </c>
+      <c r="E68" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1523,6 +1729,9 @@
         <v>2244000000</v>
       </c>
       <c r="D69" t="n">
+        <v>21</v>
+      </c>
+      <c r="E69" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1539,6 +1748,9 @@
         <v>52500000</v>
       </c>
       <c r="D70" t="n">
+        <v>3</v>
+      </c>
+      <c r="E70" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1555,6 +1767,9 @@
         <v>505300000</v>
       </c>
       <c r="D71" t="n">
+        <v>47</v>
+      </c>
+      <c r="E71" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1571,6 +1786,9 @@
         <v>26160000</v>
       </c>
       <c r="D72" t="n">
+        <v>12</v>
+      </c>
+      <c r="E72" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1587,6 +1805,9 @@
         <v>1384500000</v>
       </c>
       <c r="D73" t="n">
+        <v>13</v>
+      </c>
+      <c r="E73" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1603,7 +1824,10 @@
         <v>10845500000</v>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>60</v>
+      </c>
+      <c r="E74" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="75">
@@ -1619,6 +1843,9 @@
         <v>94600000</v>
       </c>
       <c r="D75" t="n">
+        <v>8</v>
+      </c>
+      <c r="E75" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1635,6 +1862,9 @@
         <v>66490000000</v>
       </c>
       <c r="D76" t="n">
+        <v>61</v>
+      </c>
+      <c r="E76" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1651,6 +1881,9 @@
         <v>163500000</v>
       </c>
       <c r="D77" t="n">
+        <v>3</v>
+      </c>
+      <c r="E77" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1667,6 +1900,9 @@
         <v>32700000</v>
       </c>
       <c r="D78" t="n">
+        <v>3</v>
+      </c>
+      <c r="E78" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1683,6 +1919,9 @@
         <v>152250000</v>
       </c>
       <c r="D79" t="n">
+        <v>3</v>
+      </c>
+      <c r="E79" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1699,6 +1938,9 @@
         <v>127800000</v>
       </c>
       <c r="D80" t="n">
+        <v>3</v>
+      </c>
+      <c r="E80" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1715,6 +1957,9 @@
         <v>3260700000</v>
       </c>
       <c r="D81" t="n">
+        <v>28</v>
+      </c>
+      <c r="E81" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1731,6 +1976,9 @@
         <v>640800000</v>
       </c>
       <c r="D82" t="n">
+        <v>21</v>
+      </c>
+      <c r="E82" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1747,6 +1995,9 @@
         <v>1398750000</v>
       </c>
       <c r="D83" t="n">
+        <v>11</v>
+      </c>
+      <c r="E83" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1763,6 +2014,9 @@
         <v>21300000</v>
       </c>
       <c r="D84" t="n">
+        <v>2</v>
+      </c>
+      <c r="E84" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1779,6 +2033,9 @@
         <v>3171750000</v>
       </c>
       <c r="D85" t="n">
+        <v>11</v>
+      </c>
+      <c r="E85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1795,6 +2052,9 @@
         <v>15794100000</v>
       </c>
       <c r="D86" t="n">
+        <v>12</v>
+      </c>
+      <c r="E86" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1811,7 +2071,10 @@
         <v>24605000000</v>
       </c>
       <c r="D87" t="n">
-        <v>0</v>
+        <v>50</v>
+      </c>
+      <c r="E87" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="88">
@@ -1827,6 +2090,9 @@
         <v>21800000</v>
       </c>
       <c r="D88" t="n">
+        <v>2</v>
+      </c>
+      <c r="E88" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1843,6 +2109,9 @@
         <v>606100000</v>
       </c>
       <c r="D89" t="n">
+        <v>18</v>
+      </c>
+      <c r="E89" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1859,6 +2128,9 @@
         <v>3299000000</v>
       </c>
       <c r="D90" t="n">
+        <v>26</v>
+      </c>
+      <c r="E90" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1875,6 +2147,9 @@
         <v>13341600000</v>
       </c>
       <c r="D91" t="n">
+        <v>36</v>
+      </c>
+      <c r="E91" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1891,6 +2166,9 @@
         <v>876650000</v>
       </c>
       <c r="D92" t="n">
+        <v>40</v>
+      </c>
+      <c r="E92" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1907,7 +2185,10 @@
         <v>1878600000</v>
       </c>
       <c r="D93" t="n">
-        <v>0</v>
+        <v>54</v>
+      </c>
+      <c r="E93" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="94">
@@ -1923,6 +2204,9 @@
         <v>346800000</v>
       </c>
       <c r="D94" t="n">
+        <v>40</v>
+      </c>
+      <c r="E94" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1939,6 +2223,9 @@
         <v>85200000</v>
       </c>
       <c r="D95" t="n">
+        <v>2</v>
+      </c>
+      <c r="E95" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1955,6 +2242,9 @@
         <v>308850000</v>
       </c>
       <c r="D96" t="n">
+        <v>29</v>
+      </c>
+      <c r="E96" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1971,7 +2261,10 @@
         <v>3175300000</v>
       </c>
       <c r="D97" t="n">
-        <v>0</v>
+        <v>79</v>
+      </c>
+      <c r="E97" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="98">
@@ -1987,6 +2280,9 @@
         <v>234300000</v>
       </c>
       <c r="D98" t="n">
+        <v>11</v>
+      </c>
+      <c r="E98" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2003,6 +2299,9 @@
         <v>223650000</v>
       </c>
       <c r="D99" t="n">
+        <v>7</v>
+      </c>
+      <c r="E99" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2019,6 +2318,9 @@
         <v>191700000</v>
       </c>
       <c r="D100" t="n">
+        <v>6</v>
+      </c>
+      <c r="E100" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2035,7 +2337,10 @@
         <v>2339700000</v>
       </c>
       <c r="D101" t="n">
-        <v>0</v>
+        <v>61</v>
+      </c>
+      <c r="E101" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="102">
@@ -2051,6 +2356,9 @@
         <v>1101210000</v>
       </c>
       <c r="D102" t="n">
+        <v>44</v>
+      </c>
+      <c r="E102" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2067,7 +2375,10 @@
         <v>15336000000</v>
       </c>
       <c r="D103" t="n">
-        <v>0</v>
+        <v>68</v>
+      </c>
+      <c r="E103" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="104">
@@ -2083,6 +2394,9 @@
         <v>1518750000</v>
       </c>
       <c r="D104" t="n">
+        <v>26</v>
+      </c>
+      <c r="E104" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2099,6 +2413,9 @@
         <v>182390000</v>
       </c>
       <c r="D105" t="n">
+        <v>46</v>
+      </c>
+      <c r="E105" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2115,6 +2432,9 @@
         <v>1816200000</v>
       </c>
       <c r="D106" t="n">
+        <v>6</v>
+      </c>
+      <c r="E106" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2131,6 +2451,9 @@
         <v>63083150000</v>
       </c>
       <c r="D107" t="n">
+        <v>125</v>
+      </c>
+      <c r="E107" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2147,6 +2470,9 @@
         <v>32700000</v>
       </c>
       <c r="D108" t="n">
+        <v>3</v>
+      </c>
+      <c r="E108" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2163,6 +2489,9 @@
         <v>393800000</v>
       </c>
       <c r="D109" t="n">
+        <v>10</v>
+      </c>
+      <c r="E109" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2179,6 +2508,9 @@
         <v>32700000</v>
       </c>
       <c r="D110" t="n">
+        <v>3</v>
+      </c>
+      <c r="E110" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2195,6 +2527,9 @@
         <v>49350000</v>
       </c>
       <c r="D111" t="n">
+        <v>6</v>
+      </c>
+      <c r="E111" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2211,6 +2546,9 @@
         <v>130050000</v>
       </c>
       <c r="D112" t="n">
+        <v>12</v>
+      </c>
+      <c r="E112" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2227,6 +2565,9 @@
         <v>446900000</v>
       </c>
       <c r="D113" t="n">
+        <v>7</v>
+      </c>
+      <c r="E113" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2243,7 +2584,10 @@
         <v>15796100000</v>
       </c>
       <c r="D114" t="n">
-        <v>0</v>
+        <v>65</v>
+      </c>
+      <c r="E114" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="115">
@@ -2259,6 +2603,9 @@
         <v>101400000</v>
       </c>
       <c r="D115" t="n">
+        <v>3</v>
+      </c>
+      <c r="E115" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2275,6 +2622,9 @@
         <v>65400000</v>
       </c>
       <c r="D116" t="n">
+        <v>2</v>
+      </c>
+      <c r="E116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2291,6 +2641,9 @@
         <v>1384300000</v>
       </c>
       <c r="D117" t="n">
+        <v>35</v>
+      </c>
+      <c r="E117" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2307,6 +2660,9 @@
         <v>174400000</v>
       </c>
       <c r="D118" t="n">
+        <v>8</v>
+      </c>
+      <c r="E118" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2323,6 +2679,9 @@
         <v>664900000</v>
       </c>
       <c r="D119" t="n">
+        <v>11</v>
+      </c>
+      <c r="E119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2339,6 +2698,9 @@
         <v>945000000</v>
       </c>
       <c r="D120" t="n">
+        <v>14</v>
+      </c>
+      <c r="E120" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2355,6 +2717,9 @@
         <v>386150000</v>
       </c>
       <c r="D121" t="n">
+        <v>16</v>
+      </c>
+      <c r="E121" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2371,6 +2736,9 @@
         <v>699750000</v>
       </c>
       <c r="D122" t="n">
+        <v>10</v>
+      </c>
+      <c r="E122" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2387,6 +2755,9 @@
         <v>324800000</v>
       </c>
       <c r="D123" t="n">
+        <v>4</v>
+      </c>
+      <c r="E123" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2403,7 +2774,10 @@
         <v>35970000000</v>
       </c>
       <c r="D124" t="n">
-        <v>2</v>
+        <v>33</v>
+      </c>
+      <c r="E124" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="125">
@@ -2419,6 +2793,9 @@
         <v>4883200000</v>
       </c>
       <c r="D125" t="n">
+        <v>32</v>
+      </c>
+      <c r="E125" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2435,6 +2812,9 @@
         <v>196200000</v>
       </c>
       <c r="D126" t="n">
+        <v>6</v>
+      </c>
+      <c r="E126" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2451,6 +2831,9 @@
         <v>351450000</v>
       </c>
       <c r="D127" t="n">
+        <v>6</v>
+      </c>
+      <c r="E127" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2467,6 +2850,9 @@
         <v>8773200000</v>
       </c>
       <c r="D128" t="n">
+        <v>41</v>
+      </c>
+      <c r="E128" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2483,7 +2869,10 @@
         <v>2514260000</v>
       </c>
       <c r="D129" t="n">
-        <v>0</v>
+        <v>99</v>
+      </c>
+      <c r="E129" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="130">
@@ -2499,6 +2888,9 @@
         <v>218000000</v>
       </c>
       <c r="D130" t="n">
+        <v>5</v>
+      </c>
+      <c r="E130" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2515,6 +2907,9 @@
         <v>6540000</v>
       </c>
       <c r="D131" t="n">
+        <v>3</v>
+      </c>
+      <c r="E131" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2531,7 +2926,10 @@
         <v>18706380000</v>
       </c>
       <c r="D132" t="n">
-        <v>0</v>
+        <v>89</v>
+      </c>
+      <c r="E132" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="133">
@@ -2547,6 +2945,9 @@
         <v>2250000000</v>
       </c>
       <c r="D133" t="n">
+        <v>28</v>
+      </c>
+      <c r="E133" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2563,6 +2964,9 @@
         <v>85200000</v>
       </c>
       <c r="D134" t="n">
+        <v>4</v>
+      </c>
+      <c r="E134" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2579,6 +2983,9 @@
         <v>6496000000</v>
       </c>
       <c r="D135" t="n">
+        <v>32</v>
+      </c>
+      <c r="E135" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2595,6 +3002,9 @@
         <v>24800000</v>
       </c>
       <c r="D136" t="n">
+        <v>2</v>
+      </c>
+      <c r="E136" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2611,6 +3021,9 @@
         <v>32700000</v>
       </c>
       <c r="D137" t="n">
+        <v>3</v>
+      </c>
+      <c r="E137" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2627,7 +3040,10 @@
         <v>25344050000</v>
       </c>
       <c r="D138" t="n">
-        <v>0</v>
+        <v>49</v>
+      </c>
+      <c r="E138" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="139">
@@ -2643,6 +3059,9 @@
         <v>51627000000</v>
       </c>
       <c r="D139" t="n">
+        <v>49</v>
+      </c>
+      <c r="E139" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2659,6 +3078,9 @@
         <v>127800000</v>
       </c>
       <c r="D140" t="n">
+        <v>2</v>
+      </c>
+      <c r="E140" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2675,6 +3097,9 @@
         <v>52888500000</v>
       </c>
       <c r="D141" t="n">
+        <v>102</v>
+      </c>
+      <c r="E141" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2691,6 +3116,9 @@
         <v>1597500000</v>
       </c>
       <c r="D142" t="n">
+        <v>5</v>
+      </c>
+      <c r="E142" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2707,6 +3135,9 @@
         <v>10900000</v>
       </c>
       <c r="D143" t="n">
+        <v>5</v>
+      </c>
+      <c r="E143" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2723,6 +3154,9 @@
         <v>45440000</v>
       </c>
       <c r="D144" t="n">
+        <v>8</v>
+      </c>
+      <c r="E144" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2739,6 +3173,9 @@
         <v>381500000</v>
       </c>
       <c r="D145" t="n">
+        <v>7</v>
+      </c>
+      <c r="E145" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2755,6 +3192,9 @@
         <v>2028000000</v>
       </c>
       <c r="D146" t="n">
+        <v>3</v>
+      </c>
+      <c r="E146" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2771,6 +3211,9 @@
         <v>959200000</v>
       </c>
       <c r="D147" t="n">
+        <v>11</v>
+      </c>
+      <c r="E147" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2787,6 +3230,9 @@
         <v>1278000000</v>
       </c>
       <c r="D148" t="n">
+        <v>3</v>
+      </c>
+      <c r="E148" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2803,6 +3249,9 @@
         <v>32700000</v>
       </c>
       <c r="D149" t="n">
+        <v>3</v>
+      </c>
+      <c r="E149" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2819,6 +3268,9 @@
         <v>928000000</v>
       </c>
       <c r="D150" t="n">
+        <v>16</v>
+      </c>
+      <c r="E150" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2835,6 +3287,9 @@
         <v>32700000</v>
       </c>
       <c r="D151" t="n">
+        <v>3</v>
+      </c>
+      <c r="E151" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2851,6 +3306,9 @@
         <v>105307600000</v>
       </c>
       <c r="D152" t="n">
+        <v>131</v>
+      </c>
+      <c r="E152" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2867,6 +3325,9 @@
         <v>154200000</v>
       </c>
       <c r="D153" t="n">
+        <v>12</v>
+      </c>
+      <c r="E153" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2883,6 +3344,9 @@
         <v>171650000</v>
       </c>
       <c r="D154" t="n">
+        <v>16</v>
+      </c>
+      <c r="E154" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2899,6 +3363,9 @@
         <v>71400000</v>
       </c>
       <c r="D155" t="n">
+        <v>3</v>
+      </c>
+      <c r="E155" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2915,7 +3382,10 @@
         <v>13053000000</v>
       </c>
       <c r="D156" t="n">
-        <v>0</v>
+        <v>53</v>
+      </c>
+      <c r="E156" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="157">
@@ -2931,6 +3401,9 @@
         <v>17040000000</v>
       </c>
       <c r="D157" t="n">
+        <v>40</v>
+      </c>
+      <c r="E157" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2947,6 +3420,9 @@
         <v>859400000</v>
       </c>
       <c r="D158" t="n">
+        <v>11</v>
+      </c>
+      <c r="E158" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2963,6 +3439,9 @@
         <v>127800000</v>
       </c>
       <c r="D159" t="n">
+        <v>4</v>
+      </c>
+      <c r="E159" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2979,6 +3458,9 @@
         <v>589050000</v>
       </c>
       <c r="D160" t="n">
+        <v>3</v>
+      </c>
+      <c r="E160" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2995,6 +3477,9 @@
         <v>31950000</v>
       </c>
       <c r="D161" t="n">
+        <v>3</v>
+      </c>
+      <c r="E161" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3011,6 +3496,9 @@
         <v>1341900000</v>
       </c>
       <c r="D162" t="n">
+        <v>16</v>
+      </c>
+      <c r="E162" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3027,6 +3515,9 @@
         <v>2404800000</v>
       </c>
       <c r="D163" t="n">
+        <v>24</v>
+      </c>
+      <c r="E163" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3043,6 +3534,9 @@
         <v>152250000</v>
       </c>
       <c r="D164" t="n">
+        <v>3</v>
+      </c>
+      <c r="E164" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3059,6 +3553,9 @@
         <v>130800000</v>
       </c>
       <c r="D165" t="n">
+        <v>3</v>
+      </c>
+      <c r="E165" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3075,7 +3572,10 @@
         <v>17461000000</v>
       </c>
       <c r="D166" t="n">
-        <v>0</v>
+        <v>72</v>
+      </c>
+      <c r="E166" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="167">
@@ -3091,7 +3591,10 @@
         <v>18872300000</v>
       </c>
       <c r="D167" t="n">
-        <v>0</v>
+        <v>80</v>
+      </c>
+      <c r="E167" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="168">
@@ -3107,6 +3610,9 @@
         <v>159750000</v>
       </c>
       <c r="D168" t="n">
+        <v>3</v>
+      </c>
+      <c r="E168" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3123,6 +3629,9 @@
         <v>163500000</v>
       </c>
       <c r="D169" t="n">
+        <v>3</v>
+      </c>
+      <c r="E169" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3139,6 +3648,9 @@
         <v>27690000</v>
       </c>
       <c r="D170" t="n">
+        <v>13</v>
+      </c>
+      <c r="E170" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3155,6 +3667,9 @@
         <v>275000000</v>
       </c>
       <c r="D171" t="n">
+        <v>11</v>
+      </c>
+      <c r="E171" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3171,6 +3686,9 @@
         <v>511200000</v>
       </c>
       <c r="D172" t="n">
+        <v>6</v>
+      </c>
+      <c r="E172" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3187,6 +3705,9 @@
         <v>54500000</v>
       </c>
       <c r="D173" t="n">
+        <v>5</v>
+      </c>
+      <c r="E173" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3203,6 +3724,9 @@
         <v>37200000</v>
       </c>
       <c r="D174" t="n">
+        <v>3</v>
+      </c>
+      <c r="E174" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3219,6 +3743,9 @@
         <v>2428200000</v>
       </c>
       <c r="D175" t="n">
+        <v>6</v>
+      </c>
+      <c r="E175" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3235,7 +3762,10 @@
         <v>24437570000</v>
       </c>
       <c r="D176" t="n">
-        <v>0</v>
+        <v>227</v>
+      </c>
+      <c r="E176" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="177">
@@ -3251,6 +3781,9 @@
         <v>1308000000</v>
       </c>
       <c r="D177" t="n">
+        <v>3</v>
+      </c>
+      <c r="E177" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3267,7 +3800,10 @@
         <v>6583950000</v>
       </c>
       <c r="D178" t="n">
-        <v>0</v>
+        <v>55</v>
+      </c>
+      <c r="E178" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="179">
@@ -3283,6 +3819,9 @@
         <v>65400000</v>
       </c>
       <c r="D179" t="n">
+        <v>3</v>
+      </c>
+      <c r="E179" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3299,6 +3838,9 @@
         <v>35700000</v>
       </c>
       <c r="D180" t="n">
+        <v>3</v>
+      </c>
+      <c r="E180" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3315,6 +3857,9 @@
         <v>392400000</v>
       </c>
       <c r="D181" t="n">
+        <v>18</v>
+      </c>
+      <c r="E181" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3331,6 +3876,9 @@
         <v>319500000</v>
       </c>
       <c r="D182" t="n">
+        <v>6</v>
+      </c>
+      <c r="E182" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3347,7 +3895,10 @@
         <v>138220000</v>
       </c>
       <c r="D183" t="n">
-        <v>0</v>
+        <v>59</v>
+      </c>
+      <c r="E183" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>